<commit_message>
Migrate minimal config sample to explicit authoring policy v2
</commit_message>
<xml_diff>
--- a/com.zerogamestudio.zeroengine.config-pipeline/Samples~/MinimalItemDrop/Config/drops.xlsx
+++ b/com.zerogamestudio.zeroengine.config-pipeline/Samples~/MinimalItemDrop/Config/drops.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:bookViews>
     <x:workbookView firstSheet="3" activeTab="3"/>
   </x:bookViews>
@@ -81,7 +81,7 @@
   <x:cellStyleXfs count="1">
     <x:xf/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="20">
     <x:xf/>
     <x:xf applyProtection="1">
       <x:protection locked="0"/>
@@ -108,6 +108,34 @@
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="49" applyNumberFormat="1" applyProtection="1">
+      <x:protection locked="0"/>
+    </x:xf>
+    <x:xf xfId="0"/>
+    <x:xf xfId="0" applyProtection="1">
+      <x:protection locked="0"/>
+    </x:xf>
+    <x:xf fontId="1" fillId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf fontId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf fontId="3" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="49" xfId="0" applyNumberFormat="1" applyProtection="1">
       <x:protection locked="0"/>
     </x:xf>
   </x:cellXfs>
@@ -147,312 +175,312 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="0" t="inlineStr">
+      <x:c r="A1" s="10" t="inlineStr">
         <x:is>
           <x:t>Sheet</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="0" t="inlineStr">
+      <x:c r="B1" s="10" t="inlineStr">
         <x:is>
           <x:t>Field</x:t>
         </x:is>
       </x:c>
-      <x:c r="C1" s="0" t="inlineStr">
+      <x:c r="C1" s="10" t="inlineStr">
         <x:is>
           <x:t>Title</x:t>
         </x:is>
       </x:c>
-      <x:c r="D1" s="0" t="inlineStr">
+      <x:c r="D1" s="10" t="inlineStr">
         <x:is>
           <x:t>Type</x:t>
         </x:is>
       </x:c>
-      <x:c r="E1" s="0" t="inlineStr">
+      <x:c r="E1" s="10" t="inlineStr">
         <x:is>
           <x:t>Required</x:t>
         </x:is>
       </x:c>
-      <x:c r="F1" s="0" t="inlineStr">
+      <x:c r="F1" s="10" t="inlineStr">
         <x:is>
           <x:t>Default</x:t>
         </x:is>
       </x:c>
-      <x:c r="G1" s="0" t="inlineStr">
+      <x:c r="G1" s="10" t="inlineStr">
         <x:is>
           <x:t>Range/Enum</x:t>
         </x:is>
       </x:c>
-      <x:c r="H1" s="0" t="inlineStr">
+      <x:c r="H1" s="10" t="inlineStr">
         <x:is>
           <x:t>Reference</x:t>
         </x:is>
       </x:c>
-      <x:c r="I1" s="0" t="inlineStr">
+      <x:c r="I1" s="10" t="inlineStr">
         <x:is>
           <x:t>Unit</x:t>
         </x:is>
       </x:c>
-      <x:c r="J1" s="0" t="inlineStr">
+      <x:c r="J1" s="10" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="0" t="inlineStr">
+      <x:c r="A2" s="10" t="inlineStr">
         <x:is>
           <x:t>DropTables</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="0" t="inlineStr">
+      <x:c r="B2" s="10" t="inlineStr">
         <x:is>
           <x:t>id</x:t>
         </x:is>
       </x:c>
-      <x:c r="C2" s="0" t="inlineStr">
+      <x:c r="C2" s="10" t="inlineStr">
         <x:is>
           <x:t>掉落表 ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="D2" s="0" t="inlineStr">
+      <x:c r="D2" s="10" t="inlineStr">
         <x:is>
           <x:t>string</x:t>
         </x:is>
       </x:c>
-      <x:c r="E2" s="0" t="inlineStr">
+      <x:c r="E2" s="10" t="inlineStr">
         <x:is>
           <x:t>yes</x:t>
         </x:is>
       </x:c>
-      <x:c r="F2" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="G2" s="0" t="inlineStr">
+      <x:c r="F2" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="G2" s="10" t="inlineStr">
         <x:is>
           <x:t>..</x:t>
         </x:is>
       </x:c>
-      <x:c r="H2" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="I2" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="J2" s="0" t="inlineStr">
+      <x:c r="H2" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="I2" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="J2" s="10" t="inlineStr">
         <x:is>
           <x:t/>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="0" t="inlineStr">
+      <x:c r="A3" s="10" t="inlineStr">
         <x:is>
           <x:t>DropEntries</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="0" t="inlineStr">
+      <x:c r="B3" s="10" t="inlineStr">
         <x:is>
           <x:t>id</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" s="0" t="inlineStr">
+      <x:c r="C3" s="10" t="inlineStr">
         <x:is>
           <x:t>条目 ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" s="0" t="inlineStr">
+      <x:c r="D3" s="10" t="inlineStr">
         <x:is>
           <x:t>string</x:t>
         </x:is>
       </x:c>
-      <x:c r="E3" s="0" t="inlineStr">
+      <x:c r="E3" s="10" t="inlineStr">
         <x:is>
           <x:t>yes</x:t>
         </x:is>
       </x:c>
-      <x:c r="F3" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="G3" s="0" t="inlineStr">
+      <x:c r="F3" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="G3" s="10" t="inlineStr">
         <x:is>
           <x:t>..</x:t>
         </x:is>
       </x:c>
-      <x:c r="H3" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="I3" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="J3" s="0" t="inlineStr">
+      <x:c r="H3" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="I3" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="J3" s="10" t="inlineStr">
         <x:is>
           <x:t/>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="0" t="inlineStr">
+      <x:c r="A4" s="10" t="inlineStr">
         <x:is>
           <x:t>DropEntries</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="0" t="inlineStr">
+      <x:c r="B4" s="10" t="inlineStr">
         <x:is>
           <x:t>order</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="0" t="inlineStr">
+      <x:c r="C4" s="10" t="inlineStr">
         <x:is>
           <x:t>顺序</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="0" t="inlineStr">
+      <x:c r="D4" s="10" t="inlineStr">
         <x:is>
           <x:t>int32</x:t>
         </x:is>
       </x:c>
-      <x:c r="E4" s="0" t="inlineStr">
+      <x:c r="E4" s="10" t="inlineStr">
         <x:is>
           <x:t>yes</x:t>
         </x:is>
       </x:c>
-      <x:c r="F4" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="G4" s="0" t="inlineStr">
+      <x:c r="F4" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="G4" s="10" t="inlineStr">
         <x:is>
           <x:t>0..</x:t>
         </x:is>
       </x:c>
-      <x:c r="H4" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="I4" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="J4" s="0" t="inlineStr">
+      <x:c r="H4" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="I4" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="J4" s="10" t="inlineStr">
         <x:is>
           <x:t/>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="0" t="inlineStr">
+      <x:c r="A5" s="10" t="inlineStr">
         <x:is>
           <x:t>DropEntries</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="0" t="inlineStr">
+      <x:c r="B5" s="10" t="inlineStr">
         <x:is>
           <x:t>itemId</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="0" t="inlineStr">
+      <x:c r="C5" s="10" t="inlineStr">
         <x:is>
           <x:t>物品 ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="0" t="inlineStr">
+      <x:c r="D5" s="10" t="inlineStr">
         <x:is>
           <x:t>string</x:t>
         </x:is>
       </x:c>
-      <x:c r="E5" s="0" t="inlineStr">
+      <x:c r="E5" s="10" t="inlineStr">
         <x:is>
           <x:t>yes</x:t>
         </x:is>
       </x:c>
-      <x:c r="F5" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="G5" s="0" t="inlineStr">
+      <x:c r="F5" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="10" t="inlineStr">
         <x:is>
           <x:t>..</x:t>
         </x:is>
       </x:c>
-      <x:c r="H5" s="0" t="inlineStr">
+      <x:c r="H5" s="10" t="inlineStr">
         <x:is>
           <x:t>#/properties/items/items/properties/id</x:t>
         </x:is>
       </x:c>
-      <x:c r="I5" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="J5" s="0" t="inlineStr">
+      <x:c r="I5" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="J5" s="10" t="inlineStr">
         <x:is>
           <x:t/>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="0" t="inlineStr">
+      <x:c r="A6" s="10" t="inlineStr">
         <x:is>
           <x:t>DropEntries</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="0" t="inlineStr">
+      <x:c r="B6" s="10" t="inlineStr">
         <x:is>
           <x:t>chance</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="0" t="inlineStr">
+      <x:c r="C6" s="10" t="inlineStr">
         <x:is>
           <x:t>概率</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="0" t="inlineStr">
+      <x:c r="D6" s="10" t="inlineStr">
         <x:is>
           <x:t>float32</x:t>
         </x:is>
       </x:c>
-      <x:c r="E6" s="0" t="inlineStr">
+      <x:c r="E6" s="10" t="inlineStr">
         <x:is>
           <x:t>yes</x:t>
         </x:is>
       </x:c>
-      <x:c r="F6" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="G6" s="0" t="inlineStr">
+      <x:c r="F6" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="10" t="inlineStr">
         <x:is>
           <x:t>0..1</x:t>
         </x:is>
       </x:c>
-      <x:c r="H6" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="I6" s="0" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="J6" s="0" t="inlineStr">
+      <x:c r="H6" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="I6" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="J6" s="10" t="inlineStr">
         <x:is>
           <x:t/>
         </x:is>
@@ -467,74 +495,74 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="0" t="inlineStr">
+      <x:c r="A1" s="10" t="inlineStr">
         <x:is>
           <x:t>toolFormatVersion</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="0" t="inlineStr">
+      <x:c r="B1" s="10" t="inlineStr">
         <x:is>
           <x:t>2</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="0" t="inlineStr">
+      <x:c r="A2" s="10" t="inlineStr">
         <x:is>
           <x:t>schemaId</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="0" t="inlineStr">
+      <x:c r="B2" s="10" t="inlineStr">
         <x:is>
           <x:t>urn:zgs:sample:item-drop</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="0" t="inlineStr">
+      <x:c r="A3" s="10" t="inlineStr">
         <x:is>
           <x:t>schemaVersion</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="0" t="inlineStr">
-        <x:is>
-          <x:t>1</x:t>
+      <x:c r="B3" s="10" t="inlineStr">
+        <x:is>
+          <x:t>2</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="0" t="inlineStr">
+      <x:c r="A4" s="10" t="inlineStr">
         <x:is>
           <x:t>schemaHash</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="0" t="inlineStr">
-        <x:is>
-          <x:t>801aa05b1218a88778517f78eecb6dc2fbf97b00466181dc80ad2d112b314815</x:t>
+      <x:c r="B4" s="10" t="inlineStr">
+        <x:is>
+          <x:t>af8e87178e1f71c586e1bc34119dafc54eacd3ceaa5f1e50e940ab7953af4724</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="0" t="inlineStr">
+      <x:c r="A5" s="10" t="inlineStr">
         <x:is>
           <x:t>configSetId</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="0" t="inlineStr">
+      <x:c r="B5" s="10" t="inlineStr">
         <x:is>
           <x:t>sample.item-drop</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="0" t="inlineStr">
+      <x:c r="A6" s="10" t="inlineStr">
         <x:is>
           <x:t>workbookBaseHash</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="0" t="inlineStr">
-        <x:is>
-          <x:t>f76e669736ac0938cd65fc4954e4cbfb239fcc50b451d5023fac68d66b3e845d</x:t>
+      <x:c r="B6" s="10" t="inlineStr">
+        <x:is>
+          <x:t>13255d23d0c392d6225b9b13be78d2981385d99ee84681ff7aaaadc8ee1e7cd7</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -560,85 +588,85 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="2" t="inlineStr">
+      <x:c r="A1" s="12" t="inlineStr">
         <x:is>
           <x:t>配置目录</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="3" t="inlineStr">
+      <x:c r="A2" s="13" t="inlineStr">
         <x:is>
           <x:t>点击 Sheet 名称进入配置；保存后回 Unity 执行 Check / Plan / Apply。</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="3" t="inlineStr">
+      <x:c r="A3" s="13" t="inlineStr">
         <x:is>
           <x:t>说明：标注“仅策划，不导出”或“关联键，不导出”的列不会进入运行时 JSON / DTO。</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
-      <x:c r="A4" s="4" t="inlineStr">
+      <x:c r="A4" s="14" t="inlineStr">
         <x:is>
           <x:t>配置模块</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="4" t="inlineStr">
+      <x:c r="B4" s="14" t="inlineStr">
         <x:is>
           <x:t>Sheet</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="4" t="inlineStr">
+      <x:c r="C4" s="14" t="inlineStr">
         <x:is>
           <x:t>说明</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="4" t="inlineStr">
+      <x:c r="D4" s="14" t="inlineStr">
         <x:is>
           <x:t>字段数</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="5" ht="21" customHeight="1">
-      <x:c r="A5" s="6" t="inlineStr">
+      <x:c r="A5" s="16" t="inlineStr">
         <x:is>
           <x:t>dropTables</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="5" t="inlineStr">
+      <x:c r="B5" s="15" t="inlineStr">
         <x:is>
           <x:t>DropTables</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="6" t="n">
+      <x:c r="C5" s="16" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21" customHeight="1">
-      <x:c r="A6" s="6" t="inlineStr">
+      <x:c r="A6" s="16" t="inlineStr">
         <x:is>
           <x:t>entries</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="5" t="inlineStr">
+      <x:c r="B6" s="15" t="inlineStr">
         <x:is>
           <x:t>DropEntries</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="6" t="n">
+      <x:c r="C6" s="16" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="16" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -658,27 +686,27 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:cols>
-    <x:col min="1" max="1" width="28" style="9" customWidth="1"/>
+    <x:col min="1" max="1" width="28" style="9" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" hidden="1">
-      <x:c r="A1" s="0" t="inlineStr">
+      <x:c r="A1" s="10" t="inlineStr">
         <x:is>
           <x:t>id</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="8" t="inlineStr">
+      <x:c r="A2" s="18" t="inlineStr">
         <x:is>
           <x:t>← 配置目录 ｜ ＊ 掉落表 ID</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="9" t="inlineStr">
+      <x:c r="A3" s="19" t="inlineStr">
         <x:is>
           <x:t>drop.starter</x:t>
         </x:is>
@@ -695,89 +723,89 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:cols>
     <x:col min="1" max="1" width="28" style="9" customWidth="1"/>
-    <x:col min="2" max="2" width="28" style="9" customWidth="1"/>
-    <x:col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <x:col min="4" max="4" width="22" style="9" customWidth="1"/>
-    <x:col min="5" max="5" width="15" style="1" customWidth="1"/>
+    <x:col min="2" max="2" width="28" style="9" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" style="1" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" style="9" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" style="1" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" hidden="1">
-      <x:c r="A1" s="0" t="inlineStr">
+      <x:c r="A1" s="10" t="inlineStr">
         <x:is>
           <x:t>dropTableId</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="0" t="inlineStr">
+      <x:c r="B1" s="10" t="inlineStr">
         <x:is>
           <x:t>id</x:t>
         </x:is>
       </x:c>
-      <x:c r="C1" s="0" t="inlineStr">
+      <x:c r="C1" s="10" t="inlineStr">
         <x:is>
           <x:t>order</x:t>
         </x:is>
       </x:c>
-      <x:c r="D1" s="0" t="inlineStr">
+      <x:c r="D1" s="10" t="inlineStr">
         <x:is>
           <x:t>itemId</x:t>
         </x:is>
       </x:c>
-      <x:c r="E1" s="0" t="inlineStr">
+      <x:c r="E1" s="10" t="inlineStr">
         <x:is>
           <x:t>chance</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="8" t="inlineStr">
+      <x:c r="A2" s="18" t="inlineStr">
         <x:is>
           <x:t>← 配置目录 ｜ ＊ dropTableId（关联键，不导出）</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="7" t="inlineStr">
+      <x:c r="B2" s="17" t="inlineStr">
         <x:is>
           <x:t>＊ 条目 ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="C2" s="7" t="inlineStr">
+      <x:c r="C2" s="17" t="inlineStr">
         <x:is>
           <x:t>＊ 顺序</x:t>
         </x:is>
       </x:c>
-      <x:c r="D2" s="7" t="inlineStr">
+      <x:c r="D2" s="17" t="inlineStr">
         <x:is>
           <x:t>＊ 物品 ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="E2" s="7" t="inlineStr">
+      <x:c r="E2" s="17" t="inlineStr">
         <x:is>
           <x:t>＊ 概率</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="9" t="inlineStr">
+      <x:c r="A3" s="19" t="inlineStr">
         <x:is>
           <x:t>drop.starter</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="9" t="inlineStr">
+      <x:c r="B3" s="19" t="inlineStr">
         <x:is>
           <x:t>entry.coin</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" s="1" t="n">
+      <x:c r="C3" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D3" s="9" t="inlineStr">
+      <x:c r="D3" s="19" t="inlineStr">
         <x:is>
           <x:t>item.coin</x:t>
         </x:is>
       </x:c>
-      <x:c r="E3" s="1" t="n">
+      <x:c r="E3" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>

</xml_diff>